<commit_message>
Add Excel-driven data provider for login test
</commit_message>
<xml_diff>
--- a/testData/testdatahybrid.xlsx
+++ b/testData/testdatahybrid.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\IdeaProjects\HybridFrameworkProject\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C2BAAA-0971-4ABA-AEF5-60DD57DBDD05}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF6DC69E-7506-4621-AC27-1207E973D87C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{185FB971-BC2B-4D66-9C9B-AAB735B041DB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>username</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>Laxmi</t>
+  </si>
+  <si>
+    <t>invalid</t>
   </si>
 </sst>
 </file>
@@ -549,7 +552,7 @@
         <v>9</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -582,7 +585,7 @@
         <v>16</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -593,7 +596,7 @@
         <v>18</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>